<commit_message>
Every result, table, figure and vignette from the refit on the corrected sample
The whole manifest was rerun on the 752-syndicate-year sample. What moved in the
headline: the RITC tail is probable rather than near-certain (P = 0.85, was 0.97);
the concentration slopes are unresolved where they had been reported as an effect;
Vignette 1's transfer factor falls from 0.770 to 0.333; and P(fall) reaches 0.999.
The dispersion parameters settle at k = 0.61, gamma = 0.19 and sigma = 0.021, with
the two regimes at nu = 3.10 and nu = 2.42.

results/disposition_ledger.csv and paper_pack/table39_reconciliation.tex are new: the
ledger records what happened to every corpus record between the 908 extracted and the
752 fitted, and Table 39 reconciles the two counts line by line. Both are declared
manifest outputs, so the verifier now checks them.

docs/current-results.md is regenerated from the record.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vignettes/vignette-1/decomposition_summary.xlsx
+++ b/vignettes/vignette-1/decomposition_summary.xlsx
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.07244399999999999</v>
+        <v>0.061875</v>
       </c>
       <c r="C2" t="n">
-        <v>0.067217</v>
+        <v>0.059742</v>
       </c>
       <c r="D2" t="n">
-        <v>0.06408800000000001</v>
+        <v>0.05526</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.004262</v>
+        <v>-0.002989</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.004094</v>
+        <v>-0.003626</v>
       </c>
     </row>
     <row r="3">
@@ -477,19 +477,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.766024</v>
+        <v>0.626995</v>
       </c>
       <c r="C3" t="n">
-        <v>0.408942</v>
+        <v>0.316348</v>
       </c>
       <c r="D3" t="n">
-        <v>0.38559</v>
+        <v>0.298671</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.332446</v>
+        <v>-0.298557</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.047988</v>
+        <v>-0.029766</v>
       </c>
     </row>
     <row r="4">
@@ -499,19 +499,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.865683</v>
+        <v>0.770159</v>
       </c>
       <c r="C4" t="n">
-        <v>0.646491</v>
+        <v>0.376774</v>
       </c>
       <c r="D4" t="n">
-        <v>0.601285</v>
+        <v>0.35213</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.19389</v>
+        <v>-0.377166</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.070508</v>
+        <v>-0.040864</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
R85-R106: the sample is rebuilt from the re-extracted records and the rebuilt RITC scan, and every output is regenerated from one manifest run on the 678-record working sample
The re-extraction (543 substantive record changes: line-of-business totals and
closed-year tables no longer enter a mix; a mix is admitted only when its classes
reconcile with the record's premium within 10%) and the rebuilt scanner (an
acceptance is flagged by direction and effective year; 46 corpus flags, 33 in
sample, all strong-confidence) change the working sample to 678 syndicate-years
over 118 syndicates. All 61 manifest outputs are regenerated from that sample.
The README headline, the provenance note, the FX note, the referee checks, the
generated data audit and the current-results summary follow the record; the
vignette estimator lock moves to the new centres. The suite record is committed
separately, after the clean rerun's report.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vignettes/vignette-1/decomposition_summary.xlsx
+++ b/vignettes/vignette-1/decomposition_summary.xlsx
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.063027</v>
+        <v>0.066471</v>
       </c>
       <c r="C2" t="n">
-        <v>0.060566</v>
+        <v>0.062128</v>
       </c>
       <c r="D2" t="n">
-        <v>0.057513</v>
+        <v>0.057505</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.002656</v>
+        <v>-0.004175</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.002858</v>
+        <v>-0.004791</v>
       </c>
     </row>
     <row r="3">
@@ -477,19 +477,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.63491</v>
+        <v>0.654959</v>
       </c>
       <c r="C3" t="n">
-        <v>0.285902</v>
+        <v>0.36452</v>
       </c>
       <c r="D3" t="n">
-        <v>0.280086</v>
+        <v>0.339415</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.328867</v>
+        <v>-0.275218</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.025957</v>
+        <v>-0.040326</v>
       </c>
     </row>
     <row r="4">
@@ -499,19 +499,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.774709</v>
+        <v>0.744555</v>
       </c>
       <c r="C4" t="n">
-        <v>0.379013</v>
+        <v>0.416501</v>
       </c>
       <c r="D4" t="n">
-        <v>0.357118</v>
+        <v>0.388032</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.380331</v>
+        <v>-0.304124</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.03726</v>
+        <v>-0.0524</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Guard zero maturity proxies in log-phi diagnostics
</commit_message>
<xml_diff>
--- a/vignettes/vignette-1/decomposition_summary.xlsx
+++ b/vignettes/vignette-1/decomposition_summary.xlsx
@@ -458,16 +458,16 @@
         <v>0.061784</v>
       </c>
       <c r="C2" t="n">
-        <v>0.054734</v>
+        <v>0.054782</v>
       </c>
       <c r="D2" t="n">
-        <v>0.04982</v>
+        <v>0.050274</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.006211</v>
+        <v>-0.00609</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.005753</v>
+        <v>-0.005421</v>
       </c>
     </row>
     <row r="3">
@@ -480,16 +480,16 @@
         <v>0.672434</v>
       </c>
       <c r="C3" t="n">
-        <v>0.260935</v>
+        <v>0.262011</v>
       </c>
       <c r="D3" t="n">
-        <v>0.230509</v>
+        <v>0.232207</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.361453</v>
+        <v>-0.363831</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.080472</v>
+        <v>-0.07639600000000001</v>
       </c>
     </row>
     <row r="4">
@@ -502,16 +502,16 @@
         <v>0.711338</v>
       </c>
       <c r="C4" t="n">
-        <v>0.307991</v>
+        <v>0.310576</v>
       </c>
       <c r="D4" t="n">
-        <v>0.277584</v>
+        <v>0.279905</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.351095</v>
+        <v>-0.351245</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.082659</v>
+        <v>-0.080188</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Commit the outputs of the full regeneration at af5010b
Run (a) of stage 3: reproduce.py at af5010b in a clean full-history clone (core.autocrlf=false),
Python 3.12.6, g++ and cl off PATH, PROXY_WORKERS=12, PYMC_CORES unset. All 71 manifest steps ok,
390.6 minutes, finished 6 October 2026 07:58 Brisbane.

229 files changed, every one a declared output (reproduce.declared_outputs()); 16 further declared
outputs regenerated byte-identical. This commit is the launch commit for the recorded pass, which
must reproduce these outputs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vignettes/vignette-1/decomposition_summary.xlsx
+++ b/vignettes/vignette-1/decomposition_summary.xlsx
@@ -458,13 +458,13 @@
         <v>0.060827</v>
       </c>
       <c r="C2" t="n">
-        <v>0.055481</v>
+        <v>0.055231</v>
       </c>
       <c r="D2" t="n">
-        <v>0.055481</v>
+        <v>0.055231</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.005346</v>
+        <v>-0.005596</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -477,16 +477,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.634074</v>
+        <v>0.620194</v>
       </c>
       <c r="C3" t="n">
-        <v>0.264434</v>
+        <v>0.260987</v>
       </c>
       <c r="D3" t="n">
-        <v>0.264434</v>
+        <v>0.260987</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.369639</v>
+        <v>-0.359208</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -502,13 +502,13 @@
         <v>0.711338</v>
       </c>
       <c r="C4" t="n">
-        <v>0.298916</v>
+        <v>0.295407</v>
       </c>
       <c r="D4" t="n">
-        <v>0.298916</v>
+        <v>0.295407</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.412422</v>
+        <v>-0.415931</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Regenerate the sample-dependent outputs under the primary sample (649 records)
The manifest from calibrate_dispersion.py to generate_data_audit.py, one script at a time, on the loader's primary
outcome (the 649 records of the mature-cohort construction after the exchange-rate rule and the column-free 1945
figures): the working sample, the calibrations and every check, the vignette records, the paper pack, the shipped tool
and the generated documents. fetch_h10_rates.py was not run (it needs the network; the rates are unchanged). The
headline fit now has n = 649, 118 syndicates, 10 reporting years (no 2014 record) and 34 RITC-regime records.

build_current_results.py gains the branch the regeneration needs: under the primary the composition model with the
long-tail share scores 1.6 higher by-syndicate (interval spanning zero) beside a slope resolved positive, and the open
question says so instead of refusing.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vignettes/vignette-1/decomposition_summary.xlsx
+++ b/vignettes/vignette-1/decomposition_summary.xlsx
@@ -455,16 +455,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.060882</v>
+        <v>0.059367</v>
       </c>
       <c r="C2" t="n">
-        <v>0.055168</v>
+        <v>0.054584</v>
       </c>
       <c r="D2" t="n">
-        <v>0.055168</v>
+        <v>0.054584</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.005714</v>
+        <v>-0.004783</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -480,13 +480,13 @@
         <v>0.620194</v>
       </c>
       <c r="C3" t="n">
-        <v>0.256726</v>
+        <v>0.263619</v>
       </c>
       <c r="D3" t="n">
-        <v>0.256726</v>
+        <v>0.263619</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.363469</v>
+        <v>-0.356576</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -502,13 +502,13 @@
         <v>0.711338</v>
       </c>
       <c r="C4" t="n">
-        <v>0.295054</v>
+        <v>0.330368</v>
       </c>
       <c r="D4" t="n">
-        <v>0.295054</v>
+        <v>0.330368</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.416284</v>
+        <v>-0.380969</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Regenerate the outputs on the 649-record primary sample from the pass at c84bd16
The regeneration pass ran 81 steps from a fresh core.autocrlf=false clone at c84bd16 (23 October 2026,
06:15-08:58 Brisbane). 80 succeeded; check_cohort_depth_sensitivity.py stopped on one divergence in its
u <= t-3 refit and is rerun separately. Every changed path is a declared output. docs/data-provenance.md is
merged three ways so that the round-2 paragraph added after c84bd16 stays.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vignettes/vignette-1/decomposition_summary.xlsx
+++ b/vignettes/vignette-1/decomposition_summary.xlsx
@@ -458,13 +458,13 @@
         <v>0.059367</v>
       </c>
       <c r="C2" t="n">
-        <v>0.054584</v>
+        <v>0.054603</v>
       </c>
       <c r="D2" t="n">
-        <v>0.054584</v>
+        <v>0.054603</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.004783</v>
+        <v>-0.004765</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -480,13 +480,13 @@
         <v>0.620194</v>
       </c>
       <c r="C3" t="n">
-        <v>0.263619</v>
+        <v>0.263815</v>
       </c>
       <c r="D3" t="n">
-        <v>0.263619</v>
+        <v>0.263815</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.356576</v>
+        <v>-0.356379</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -502,13 +502,13 @@
         <v>0.711338</v>
       </c>
       <c r="C4" t="n">
-        <v>0.330368</v>
+        <v>0.33048</v>
       </c>
       <c r="D4" t="n">
-        <v>0.330368</v>
+        <v>0.33048</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.380969</v>
+        <v>-0.380857</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Regenerate the outputs on the 643-record primary from the pass at 4f99471
The regeneration pass ran 81 steps from a fresh core.autocrlf=false clone at 4f99471 (23 October 2026, 19:02-21:48
Brisbane), with no g++, gcc or cl on PATH, an empty TEMP, PROXY_WORKERS=12 and PYMC_CORES unset. 80 succeeded;
check_margin_sensitivity.py stopped because a size stratum held fewer unflagged syndicates than the margin variant
leaves out, and is fixed and rerun separately. Every changed path is a declared output (README.md is declared since
c83cbaf).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vignettes/vignette-1/decomposition_summary.xlsx
+++ b/vignettes/vignette-1/decomposition_summary.xlsx
@@ -455,16 +455,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.059367</v>
+        <v>0.058745</v>
       </c>
       <c r="C2" t="n">
-        <v>0.054603</v>
+        <v>0.054064</v>
       </c>
       <c r="D2" t="n">
-        <v>0.054603</v>
+        <v>0.054064</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.004765</v>
+        <v>-0.004681</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -480,13 +480,13 @@
         <v>0.620194</v>
       </c>
       <c r="C3" t="n">
-        <v>0.263815</v>
+        <v>0.266966</v>
       </c>
       <c r="D3" t="n">
-        <v>0.263815</v>
+        <v>0.266966</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.356379</v>
+        <v>-0.353228</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -502,13 +502,13 @@
         <v>0.711338</v>
       </c>
       <c r="C4" t="n">
-        <v>0.33048</v>
+        <v>0.334027</v>
       </c>
       <c r="D4" t="n">
-        <v>0.33048</v>
+        <v>0.334027</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.380857</v>
+        <v>-0.37731</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Regenerate every output on the round-8 primary (780/2016 in, 2232/2017 out)
The regeneration pass of fda5d4c (D:\tmp\r62\ocp7, 81 steps, 07:53 to 11:31 Brisbane, 24 October
2026) rewrites the outputs for final review 2's fixes: rule 4b and the incurred-first accounts
test, 780/2016 returned to the primary under rule 6, 2232/2017 and 4747/2024 out under rule 4b
(643 records, 118 syndicates, 33 RITC; 39 least-certain), the margin record control's computed
caveat, the gamma-free fit's unrounded gap column and the 50m-1bn count. Only declared outputs
changed (take_regen_outputs.py); docs/data-provenance.md is merged three ways. No fit in the pass
needed a retry.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vignettes/vignette-1/decomposition_summary.xlsx
+++ b/vignettes/vignette-1/decomposition_summary.xlsx
@@ -455,16 +455,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.058745</v>
+        <v>0.058836</v>
       </c>
       <c r="C2" t="n">
-        <v>0.054064</v>
+        <v>0.054413</v>
       </c>
       <c r="D2" t="n">
-        <v>0.054064</v>
+        <v>0.054413</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.004681</v>
+        <v>-0.004424</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -480,13 +480,13 @@
         <v>0.620194</v>
       </c>
       <c r="C3" t="n">
-        <v>0.266966</v>
+        <v>0.267257</v>
       </c>
       <c r="D3" t="n">
-        <v>0.266966</v>
+        <v>0.267257</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.353228</v>
+        <v>-0.352938</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -502,13 +502,13 @@
         <v>0.711338</v>
       </c>
       <c r="C4" t="n">
-        <v>0.334027</v>
+        <v>0.334312</v>
       </c>
       <c r="D4" t="n">
-        <v>0.334027</v>
+        <v>0.334312</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.37731</v>
+        <v>-0.377026</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Regenerate every output on the census primary (632 records, rule 8)
The regeneration pass of f6e787b (D:\tmp\r62\ocp10, 84 steps, 16:56 to 20:03 Brisbane, 26
October 2026) rewrites the outputs for the source-history rule's census (11 records set
aside; 632 records, 117 syndicates, 27 assumed-business records), the corrections to
3330/2017 and 3330/2018, the reversal of 1609/2024, the cohort-depth repairs, the frozen fold
map, the donor pool built from the loader's file, and three new producers (the small-book
diagnosis, the exclusion influence sensitivities with 33 fits, and the uncertainty figure).
Only declared outputs changed; the copy back verified 239 of 239 copied paths against the
clone, and docs/data-provenance.md is merged three ways. No fit needed a retry.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vignettes/vignette-1/decomposition_summary.xlsx
+++ b/vignettes/vignette-1/decomposition_summary.xlsx
@@ -455,16 +455,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.058836</v>
+        <v>0.058745</v>
       </c>
       <c r="C2" t="n">
-        <v>0.054413</v>
+        <v>0.054108</v>
       </c>
       <c r="D2" t="n">
-        <v>0.054413</v>
+        <v>0.054108</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.004424</v>
+        <v>-0.004638</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -477,16 +477,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.620194</v>
+        <v>0.6049369999999999</v>
       </c>
       <c r="C3" t="n">
-        <v>0.267257</v>
+        <v>0.276042</v>
       </c>
       <c r="D3" t="n">
-        <v>0.267257</v>
+        <v>0.276042</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.352938</v>
+        <v>-0.328895</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -499,16 +499,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.711338</v>
+        <v>0.672434</v>
       </c>
       <c r="C4" t="n">
-        <v>0.334312</v>
+        <v>0.3424</v>
       </c>
       <c r="D4" t="n">
-        <v>0.334312</v>
+        <v>0.3424</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.377026</v>
+        <v>-0.330034</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>

</xml_diff>